<commit_message>
Columns on home page
Automated migration updates generated by Experience Modernization Agent.

Changed files (6):
- tools/importer/import-menu-page.bundle.js
- tools/importer/import-menu-page.js
- tools/importer/page-templates.json
- tools/importer/parsers/columns-service.js
- tools/importer/reports/import-menu-page.report.xlsx
- tools/importer/reports/menu-eng.report.json
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-menu-page.report.xlsx
+++ b/tools/importer/reports/import-menu-page.report.xlsx
@@ -40,7 +40,7 @@
     <t>menu-eng.report.json</t>
   </si>
   <si>
-    <t>["columns-intro","columns-news","cards-feature","cards-feature","cards-feature","cards-feature","cards-feature","columns-service","cards-doormat","cards-doormat","cards-doormat","cards-doormat","cards-doormat","cards-doormat","cards-doormat","cards-doormat","cards-doormat","cards-doormat","cards-doormat","cards-doormat","cards-doormat","columns-links","columns-links"]</t>
+    <t>["columns-intro","columns-news","cards-feature","cards-feature","cards-feature","cards-feature","cards-feature","columns-service","columns-links","columns-links"]</t>
   </si>
   <si>
     <t>menu-eng</t>
@@ -52,7 +52,7 @@
     <t>menu-page</t>
   </si>
   <si>
-    <t>2026-04-22T18:35:20.489Z</t>
+    <t>2026-04-22T18:48:37.390Z</t>
   </si>
   <si>
     <t>Canada Border Services Agency</t>

</xml_diff>

<commit_message>
More content to blocks, initial style
Automated migration updates generated by Experience Modernization Agent.

Changed files (16):
- blocks/cards-feature/cards-feature.css
- blocks/cards-leadership/cards-leadership.css
- blocks/cards-leadership/cards-leadership.js
- blocks/columns-intro/columns-intro.css
- blocks/columns-links/columns-links.css
- blocks/columns-news/columns-news.css
- blocks/columns-service/columns-service.css
- head.html
- styles/fonts.css
- styles/styles.css
- tools/importer/import-menu-page.bundle.js
- tools/importer/import-menu-page.js
- tools/importer/page-templates.json
- tools/importer/parsers/cards-leadership.js
- tools/importer/reports/import-menu-page.report.xlsx
- tools/importer/reports/menu-eng.report.json
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-menu-page.report.xlsx
+++ b/tools/importer/reports/import-menu-page.report.xlsx
@@ -40,7 +40,7 @@
     <t>menu-eng.report.json</t>
   </si>
   <si>
-    <t>["columns-intro","columns-news","cards-feature","cards-feature","cards-feature","cards-feature","cards-feature","columns-service","columns-links","columns-links"]</t>
+    <t>["columns-intro","columns-news","cards-leadership","cards-feature","cards-feature","columns-service","columns-links","columns-links","columns-links","columns-links","columns-links"]</t>
   </si>
   <si>
     <t>menu-eng</t>
@@ -52,7 +52,7 @@
     <t>menu-page</t>
   </si>
   <si>
-    <t>2026-04-22T18:48:37.390Z</t>
+    <t>2026-04-22T19:05:41.695Z</t>
   </si>
   <si>
     <t>Canada Border Services Agency</t>

</xml_diff>

<commit_message>
Style + social links
Automated migration updates generated by Experience Modernization Agent.

Changed files (8):
- blocks/columns-intro/columns-intro.js
- blocks/columns-news/columns-news.css
- tools/importer/import-menu-page.bundle.js
- tools/importer/import-menu-page.js
- tools/importer/page-templates.json
- tools/importer/parsers/cards-feature.js
- tools/importer/reports/import-menu-page.report.xlsx
- tools/importer/reports/menu-eng.report.json
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-menu-page.report.xlsx
+++ b/tools/importer/reports/import-menu-page.report.xlsx
@@ -40,7 +40,7 @@
     <t>menu-eng.report.json</t>
   </si>
   <si>
-    <t>["columns-intro","columns-news","cards-leadership","cards-feature","cards-feature","columns-service","columns-links","columns-links","columns-links","columns-links","columns-links"]</t>
+    <t>["columns-intro","columns-news","cards-leadership","cards-feature","columns-service","columns-links","columns-links","columns-links","columns-links","columns-links"]</t>
   </si>
   <si>
     <t>menu-eng</t>
@@ -52,7 +52,7 @@
     <t>menu-page</t>
   </si>
   <si>
-    <t>2026-04-22T19:05:41.695Z</t>
+    <t>2026-04-22T19:10:28.929Z</t>
   </si>
   <si>
     <t>Canada Border Services Agency</t>

</xml_diff>